<commit_message>
Iniciação do documento tabelado padrão
</commit_message>
<xml_diff>
--- a/resultados_cnj.xlsx
+++ b/resultados_cnj.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,20 +436,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Subtítulo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
@@ -458,513 +463,608 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos) Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>1º Grau1º Grau</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>108,62%</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2025-11-28 10:59</t>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos) Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Turma RecursalTurma Recursal</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>104,28%</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2025-11-28 10:59</t>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:09</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos) Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Juizado EspecialJuizado Especial</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>101,10%</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2025-11-28 10:59</t>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:09</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos) Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>2º Grau2º Grau</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>93,29%</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2025-11-28 10:59</t>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:09</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos) Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 100% dos processos distribuídos até 31/12/2018. Tribunal Superior do Trabalho: 100% dos processos distribuídos até 31/12/2019. Justiça Estadual: pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais. Justiça Federal: todos os processos distribuídos há 16 anos (2009), 85% dos processos distribuídos até 31/12/2021 no 1º e 2º grau e 100% dos processos distribuídos até 31/12/2022 nos Juizados Especiais Federais e nas Turmas Recursais. Justiça do Trabalho: pelo menos, 94% dos processos distribuídos até 31/12/2023, nos 1º e 2º graus e 100% dos processos pendentes de julgamento há 5 anos (2020) ou mais. Justiça Eleitoral: 70% dos processos distribuídos até 31/12/2023 e todos os processos de conhecimento pendentes de julgamento há 6 anos (2019) ou mais. Justiça Militar da União: todos os processos de conhecimento pendentes de julgamento há 5 anos (2020) ou mais e 95% dos processos distribuídos até 31/12/2022 nas Auditorias e 99% dos processos distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: todos os processos de conhecimento pendentes de julgamento há 3 anos (2022) ou mais e 90% dos processos distribuídos até 31/12/2023 nas Auditorias, e 95% dos processos distribuídos até 31/12/2024 no 2º grau.</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>1º Grau1º Grau</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>106,49%</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2025-11-28 10:59</t>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos) Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 100% dos processos distribuídos até 31/12/2018. Tribunal Superior do Trabalho: 100% dos processos distribuídos até 31/12/2019. Justiça Estadual: pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais. Justiça Federal: todos os processos distribuídos há 16 anos (2009), 85% dos processos distribuídos até 31/12/2021 no 1º e 2º grau e 100% dos processos distribuídos até 31/12/2022 nos Juizados Especiais Federais e nas Turmas Recursais. Justiça do Trabalho: pelo menos, 94% dos processos distribuídos até 31/12/2023, nos 1º e 2º graus e 100% dos processos pendentes de julgamento há 5 anos (2020) ou mais. Justiça Eleitoral: 70% dos processos distribuídos até 31/12/2023 e todos os processos de conhecimento pendentes de julgamento há 6 anos (2019) ou mais. Justiça Militar da União: todos os processos de conhecimento pendentes de julgamento há 5 anos (2020) ou mais e 95% dos processos distribuídos até 31/12/2022 nas Auditorias e 99% dos processos distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: todos os processos de conhecimento pendentes de julgamento há 3 anos (2022) ou mais e 90% dos processos distribuídos até 31/12/2023 nas Auditorias, e 95% dos processos distribuídos até 31/12/2024 no 2º grau.</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>2º Grau2º Grau</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>108,61%</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2025-11-28 10:59</t>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos) Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 100% dos processos distribuídos até 31/12/2018. Tribunal Superior do Trabalho: 100% dos processos distribuídos até 31/12/2019. Justiça Estadual: pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais. Justiça Federal: todos os processos distribuídos há 16 anos (2009), 85% dos processos distribuídos até 31/12/2021 no 1º e 2º grau e 100% dos processos distribuídos até 31/12/2022 nos Juizados Especiais Federais e nas Turmas Recursais. Justiça do Trabalho: pelo menos, 94% dos processos distribuídos até 31/12/2023, nos 1º e 2º graus e 100% dos processos pendentes de julgamento há 5 anos (2020) ou mais. Justiça Eleitoral: 70% dos processos distribuídos até 31/12/2023 e todos os processos de conhecimento pendentes de julgamento há 6 anos (2019) ou mais. Justiça Militar da União: todos os processos de conhecimento pendentes de julgamento há 5 anos (2020) ou mais e 95% dos processos distribuídos até 31/12/2022 nas Auditorias e 99% dos processos distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: todos os processos de conhecimento pendentes de julgamento há 3 anos (2022) ou mais e 90% dos processos distribuídos até 31/12/2023 nas Auditorias, e 95% dos processos distribuídos até 31/12/2024 no 2º grau.</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Juizado EspecialJuizado Especial</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>98,04%</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2025-11-28 10:59</t>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:10</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos) Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 100% dos processos distribuídos até 31/12/2018. Tribunal Superior do Trabalho: 100% dos processos distribuídos até 31/12/2019. Justiça Estadual: pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais. Justiça Federal: todos os processos distribuídos há 16 anos (2009), 85% dos processos distribuídos até 31/12/2021 no 1º e 2º grau e 100% dos processos distribuídos até 31/12/2022 nos Juizados Especiais Federais e nas Turmas Recursais. Justiça do Trabalho: pelo menos, 94% dos processos distribuídos até 31/12/2023, nos 1º e 2º graus e 100% dos processos pendentes de julgamento há 5 anos (2020) ou mais. Justiça Eleitoral: 70% dos processos distribuídos até 31/12/2023 e todos os processos de conhecimento pendentes de julgamento há 6 anos (2019) ou mais. Justiça Militar da União: todos os processos de conhecimento pendentes de julgamento há 5 anos (2020) ou mais e 95% dos processos distribuídos até 31/12/2022 nas Auditorias e 99% dos processos distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: todos os processos de conhecimento pendentes de julgamento há 3 anos (2022) ou mais e 90% dos processos distribuídos até 31/12/2023 nas Auditorias, e 95% dos processos distribuídos até 31/12/2024 no 2º grau.</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Turma RecursalTurma Recursal</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>100,77%</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2025-11-28 10:59</t>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:10</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Meta 3 – Estimular a conciliação Justiça Estadual: Aumentar o indicador Índice de Conciliação do Justiça em Números em 1 ponto percentual em relação a 2024. Cláusula de barreira: 17% de Índice de Conciliação. Justiça Federal: Aumentar o Índice de Conciliação do Justiça em Números em 0,5 ponto percentual em relação ao biênio 2023/2024. Cláusula de barreira: 8% de Índice de Conciliação. Justiça do Trabalho: Aumentar o índice de conciliação em 0,5 ponto percentual em relação à média do biênio 2022/2023 ou alcançar, no mínimo, 38% de conciliação.</t>
+          <t>Meta 3 – Estimular a conciliação</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Aumentar o indicador Índice de Conciliação do Justiça em Números em 1 ponto percentual em relação a 2024. Cláusula de barreira: 17% de Índice de Conciliação.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>100,00%</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:00</t>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais Superior Tribunal de Justiça: Identificar e julgar até 31/12/2025, 90% das ações de improbidade administrativa e das ações penais relacionadas aos crimes contra a Administração Pública distribuídas até 31/12/2023 e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Estadual: Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Federal: Identificar e julgar até 31/12/2025, 70% das ações de improbidade administrativa e das ações penais relacionadas aos crimes contra a administração pública distribuídas até 31/12/2022 e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Eleitoral: Identificar e julgar até 31/12/2025, 90% dos processos referentes às eleições de 2022 e 50% dos processos referentes às eleições de 2024, distribuídos até 31/12/2024, que possam importar na perda de mandato eletivo ou em inelegibilidade.  Justiça Militar da União: Identificar e julgar até 31/12/2025, 95% dos processos da meta distribuídos até 31/12/2022 nas Auditorias e 99% dos processos da meta distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: Identificar e julgar até 31/12/2025, 95% das ações penais relacionadas aos crimes contra a Administração Pública, abrangendo, inclusive, a Lei 13.491/17, distribuídas até 31/12/2023 no 1º grau, e pelo menos 95% das distribuídas no 2º grau até 31/12/2024.</t>
+          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>Total Real</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>140,04%</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:00</t>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais Superior Tribunal de Justiça: Identificar e julgar até 31/12/2025, 90% das ações de improbidade administrativa e das ações penais relacionadas aos crimes contra a Administração Pública distribuídas até 31/12/2023 e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Estadual: Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Federal: Identificar e julgar até 31/12/2025, 70% das ações de improbidade administrativa e das ações penais relacionadas aos crimes contra a administração pública distribuídas até 31/12/2022 e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Eleitoral: Identificar e julgar até 31/12/2025, 90% dos processos referentes às eleições de 2022 e 50% dos processos referentes às eleições de 2024, distribuídos até 31/12/2024, que possam importar na perda de mandato eletivo ou em inelegibilidade.  Justiça Militar da União: Identificar e julgar até 31/12/2025, 95% dos processos da meta distribuídos até 31/12/2022 nas Auditorias e 99% dos processos da meta distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: Identificar e julgar até 31/12/2025, 95% das ações penais relacionadas aos crimes contra a Administração Pública, abrangendo, inclusive, a Lei 13.491/17, distribuídas até 31/12/2023 no 1º grau, e pelo menos 95% das distribuídas no 2º grau até 31/12/2024.</t>
+          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>Total Submeta</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>73,19%</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:00</t>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Meta 5 – Reduzir a taxa de congestionamento Superior Tribunal de Justiça: Reduzir em 0,5 ponto percentual, até 31/12/2025, a taxa de congestionamento dos processos no Superior Tribunal de Justiça, referente ao apurado em 2024. Tribunal Superior do Trabalho: Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida, exceto execuções fiscais, em relação a 2024.  Justiça Federal: Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida, exceto execuções fiscais, em relação a 2024. Cláusula de barreira: 43%. Justiça do Trabalho: Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida, exceto execuções fiscais, em relação a 2024. Cláusula de barreira na fase de conhecimento: 40%. Cláusula de barreira na fase de execução: 65%. Justiça Estadual: Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%. Justiça Militar da União: Reduzir, no mínimo, em 0,5 ponto percentual a taxa de congestionamento líquida na fase de conhecimento no 1º grau, em relação a 2024. Justiça Militar Estadual: Reduzir, no mínimo, em 0,5 ponto percentual a taxa de congestionamento líquida na fase de conhecimento no 1º grau, em relação a 2023.</t>
+          <t>Meta 5 – Reduzir a taxa de congestionamento</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>88,83%</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:00</t>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Meta 6 – Priorizar o julgamento das ações ambientais Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 75% dos processos relacionados às ações ambientais distribuídos até 31/12/2024. Justiça Estadual: 50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024. Justiça Federal: FAIXA 1 (TRF1 e TRF6): 25% dos processos que tenham por objeto matéria ambiental, distribuídos até 31/12/2024. FAIXA 2 (TRF2, TRF3, TRF4 e TRF5): 35% dos processos que tenham por objeto matéria ambiental, distribuídos até 31/12/2024.</t>
+          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>84,76%</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:00</t>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:11</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas  Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 75% dos processos relacionados aos direitos das comunidades indígenas e 75% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024. Justiça Estadual: 50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024. Justiça Federal: - FAIXA 1 (TRF1 e TRF6): 25% dos processos relacionados aos direitos das comunidades indígenas e 25% dos processos relacionados aos direitos das comunidades quilombolas, distribuídos até 31/12/2024. - FAIXA 2 (TRF2, TRF3, TRF4 e TRF5): 35% dos processos relacionados aos direitos das comunidades indígenas e 35% dos processos relacionados aos direitos das comunidades quilombolas, distribuídos até 31/12/2024.</t>
+          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>Total Indígenas</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>120,00%</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:01</t>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:11</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas  Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 75% dos processos relacionados aos direitos das comunidades indígenas e 75% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024. Justiça Estadual: 50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024. Justiça Federal: - FAIXA 1 (TRF1 e TRF6): 25% dos processos relacionados aos direitos das comunidades indígenas e 25% dos processos relacionados aos direitos das comunidades quilombolas, distribuídos até 31/12/2024. - FAIXA 2 (TRF2, TRF3, TRF4 e TRF5): 35% dos processos relacionados aos direitos das comunidades indígenas e 35% dos processos relacionados aos direitos das comunidades quilombolas, distribuídos até 31/12/2024.</t>
+          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>Total Quilombola</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>100,00%</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:01</t>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:11</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres Identificar e julgar, até 31/12/2025: Superior Tribunal de Justiça: 100% dos casos de feminicídio e de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023. Justiça Estadual: 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar, até 31/12/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>Total Violência Doméstica</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>91,31%</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:01</t>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:11</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres Identificar e julgar, até 31/12/2025: Superior Tribunal de Justiça: 100% dos casos de feminicídio e de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023. Justiça Estadual: 75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar, até 31/12/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>Total Feminicídio</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>108,62%</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:01</t>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:11</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Meta 10 – Promover os direitos da criança e do adolescente. Superior Tribunal de Justiça: Julgar 100% dos casos de sequestro internacional de crianças, distribuídos até 31/12/2024. Justiça do Trabalho: Promover, no âmbito do Programa de Combate ao Trabalho Infantil e Estímulo à Aprendizagem, pelo menos uma ação de combate ao trabalho infantil e de estímulo à aprendizagem, preferencialmente, voltada à promoção da equidade racial, de gênero ou diversidade do público-alvo, por meio do estabelecimento de parcerias interinstitucionais. Justiça Estadual: Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias. Justiça Federal: Identificar e julgar, até 31/12/2025, 100% dos casos de subtração internacional de crianças distribuídos até 31/12/2024, em cada uma das instâncias.</t>
+          <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>Total 1º Grau</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>86,57%</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:01</t>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:11</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Meta 10 – Promover os direitos da criança e do adolescente. Superior Tribunal de Justiça: Julgar 100% dos casos de sequestro internacional de crianças, distribuídos até 31/12/2024. Justiça do Trabalho: Promover, no âmbito do Programa de Combate ao Trabalho Infantil e Estímulo à Aprendizagem, pelo menos uma ação de combate ao trabalho infantil e de estímulo à aprendizagem, preferencialmente, voltada à promoção da equidade racial, de gênero ou diversidade do público-alvo, por meio do estabelecimento de parcerias interinstitucionais. Justiça Estadual: Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias. Justiça Federal: Identificar e julgar, até 31/12/2025, 100% dos casos de subtração internacional de crianças distribuídos até 31/12/2024, em cada uma das instâncias.</t>
+          <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>Total 2º Grau</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>85,09%</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2025-11-28 11:01</t>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2025-11-28 14:11</t>
         </is>
       </c>
     </row>

</xml_diff>